<commit_message>
Fix Wenjuanxing Excel format to match official 7-column template
Co-authored-by: Alanc0414 <Alanc0414@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CMport_问卷星导入_Day1.xlsx
+++ b/CMport_问卷星导入_Day1.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="试题" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,30 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="微软雅黑"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -56,32 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,540 +413,397 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>题型</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>题干</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>选项A</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>选项B</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>选项C</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>选项D</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>选项E</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>选项F</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>正确答案</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>分值</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>答案解析</t>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>解析</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>单选题</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>香港正式回归中国、香港特别行政区宣告成立的日期是？</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>1997年6月30日</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>1997年7月1日</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>1999年7月1日</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>1997年8月1日</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>【依据】历史档案/《中英联合声明》
-1997年7月1日零时，中英两国完成政权交接，中国对香港恢复行使主权，香港特别行政区正式成立。</t>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>【依据】历史档案/《中英联合声明》 1997年7月1日零时，中英两国完成政权交接，中国对香港恢复行使主权，香港特别行政区正式成立。</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>单选题</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>中英两国政府正式签署《中英联合声明》的年份是？</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>1982年</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>1984年</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>1986年</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>1990年</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>【依据】《中英联合声明》（1984年12月19日签署）
-1984年12月19日，国务院总理赵紫阳与英国首相撒切尔夫人在北京签署《中英联合声明》，确定了香港回归的法律基础。</t>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>【依据】《中英联合声明》（1984年12月19日签署） 1984年12月19日，国务院总理赵紫阳与英国首相撒切尔夫人在北京签署《中英联合声明》，确定了香港回归的法律基础。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>单选题</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>"一国两制"伟大构想的提出者是？</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>毛泽东</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>周恩来</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>邓小平</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>江泽民</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>【依据】邓小平系列讲话（1982年起）
-"一国两制"由邓小平同志创造性提出，体现了解决历史遗留问题的政治智慧，并在香港成功实践。</t>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>【依据】邓小平系列讲话（1982年起） "一国两制"由邓小平同志创造性提出，体现了解决历史遗留问题的政治智慧，并在香港成功实践。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>单选题</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>香港特别行政区区旗的主体图案是什么？</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>红底白色五星</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>红底白色洋紫荆花</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>白底红色紫荆花</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>黄底红色紫荆花</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>【依据】《香港特别行政区基本法》附件/区旗区徽条例
-香港区旗为红底，中央绘有五星花蕊的白色洋紫荆花图案，象征香港是祖国大家庭的一员。</t>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>【依据】《香港特别行政区基本法》附件/区旗区徽条例 香港区旗为红底，中央绘有五星花蕊的白色洋紫荆花图案，象征香港是祖国大家庭的一员。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>单选题</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>根据《基本法》，香港保持原有资本主义制度"五十年不变"，具体是指哪个时间段？</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>1984年至2034年</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>1997年至2047年</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>1990年至2040年</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>1997年至2050年</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>【依据】《香港特别行政区基本法》第五条
-基本法第五条明确规定，香港保持原有资本主义制度和生活方式，五十年不变，即自1997年起至2047年止。</t>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>【依据】《香港特别行政区基本法》第五条 基本法第五条明确规定，香港保持原有资本主义制度和生活方式，五十年不变，即自1997年起至2047年止。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>单选题</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>香港特别行政区第一任行政长官是谁？</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>曾荫权</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>梁振英</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>董建华</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>林郑月娥</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>【依据】历史记录
-董建华于1997年7月1日就任香港特别行政区首任行政长官，任期至2005年。</t>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>【依据】历史记录 董建华于1997年7月1日就任香港特别行政区首任行政长官，任期至2005年。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>多选题</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>《中英联合声明》的主要内容包括以下哪些？（多选）</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>《中英联合声明》的主要内容包括以下哪些？（多选）[多选题]</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>中国于1997年7月1日对香港恢复行使主权</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>英国于1997年7月1日将香港交还中国</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>香港回归后实行"一国两制"，保持现行制度五十年不变</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>英国可在香港保留军事基地50年</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>【依据】《中英联合声明》（1984年）
-联合声明确立了主权移交时间、"一国两制"政策及制度不变承诺。D项错误，回归后防务由中国负责，英方不保留军事基地。</t>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>【依据】《中英联合声明》（1984年） 联合声明确立了主权移交时间、"一国两制"政策及制度不变承诺。D项错误，回归后防务由中国负责，英方不保留军事基地。</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>多选题</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>以下关于香港特别行政区的描述，正确的是？（多选）</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>以下关于香港特别行政区的描述，正确的是？（多选）[多选题]</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>香港位于中国南部，珠江口以东</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>香港由香港岛、九龙和新界三大部分组成</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>香港是中国唯一的特别行政区</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>香港是全球重要的金融、贸易及航运中心</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>ABD</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>【依据】《香港特别行政区基本法》；地理知识
-香港由三大地理区域组成，位于珠江口东岸，是国际金融中心。C项错误，澳门也是特别行政区。</t>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>【依据】《香港特别行政区基本法》；地理知识 香港由三大地理区域组成，位于珠江口东岸，是国际金融中心。C项错误，澳门也是特别行政区。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>多选题</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>根据《基本法》，以下哪些是香港特别行政区依法享有的高度自治权？（多选）</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>根据《基本法》，以下哪些是香港特别行政区依法享有的高度自治权？（多选）[多选题]</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>独立的司法权和终审权</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>行政管理权</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>立法权</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>以"中国香港"名义参与相关国际组织和活动</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>ABCD</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>【依据】《香港特别行政区基本法》第二条、第十六条、第十七条、第十九条
-基本法第二条授权香港享有高度自治权，涵盖行政、立法、司法及对外事务等各方面。</t>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>【依据】《香港特别行政区基本法》第二条、第十六条、第十七条、第十九条 基本法第二条授权香港享有高度自治权，涵盖行政、立法、司法及对外事务等各方面。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>多项填空</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>香港特别行政区于{1997}年{7}月{1}日正式成立，是中华人民共和国的一个享有高度自治权的{特别}行政区。</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
         <is>
           <t>1997;7;1;特别</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>【依据】《香港特别行政区基本法》第一条
-基本法第一条明确指出，香港特别行政区是中华人民共和国不可分离的部分，享有高度自治权。</t>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>【依据】《香港特别行政区基本法》第一条 基本法第一条明确指出，香港特别行政区是中华人民共和国不可分离的部分，享有高度自治权。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Q7 multi-choice format for Wenjuanxing Excel import
Co-authored-by: Alanc0414 <Alanc0414@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CMport_问卷星导入_Day1.xlsx
+++ b/CMport_问卷星导入_Day1.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>【依据】历史档案/《中英联合声明》 1997年7月1日零时，中英两国完成政权交接，中国对香港恢复行使主权，香港特别行政区正式成立。</t>
+          <t>依据：历史档案/《中英联合声明》。1997年7月1日零时，中英两国完成政权交接，中国对香港恢复行使主权，香港特别行政区正式成立。</t>
         </is>
       </c>
     </row>
@@ -523,14 +523,14 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>【依据】《中英联合声明》（1984年12月19日签署） 1984年12月19日，国务院总理赵紫阳与英国首相撒切尔夫人在北京签署《中英联合声明》，确定了香港回归的法律基础。</t>
+          <t>依据：《中英联合声明》（1984年12月19日签署）。1984年12月19日，国务院总理赵紫阳与英国首相撒切尔夫人在北京签署《中英联合声明》，确定了香港回归的法律基础。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>"一国两制"伟大构想的提出者是？</t>
+          <t>一国两制伟大构想的提出者是？</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>【依据】邓小平系列讲话（1982年起） "一国两制"由邓小平同志创造性提出，体现了解决历史遗留问题的政治智慧，并在香港成功实践。</t>
+          <t>依据：邓小平系列讲话（1982年起）。一国两制由邓小平同志创造性提出，体现了解决历史遗留问题的政治智慧，并在香港成功实践。</t>
         </is>
       </c>
     </row>
@@ -597,14 +597,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>【依据】《香港特别行政区基本法》附件/区旗区徽条例 香港区旗为红底，中央绘有五星花蕊的白色洋紫荆花图案，象征香港是祖国大家庭的一员。</t>
+          <t>依据：《香港特别行政区基本法》附件/区旗区徽条例。香港区旗为红底，中央绘有五星花蕊的白色洋紫荆花图案，象征香港是祖国大家庭的一员。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>根据《基本法》，香港保持原有资本主义制度"五十年不变"，具体是指哪个时间段？</t>
+          <t>根据《基本法》，香港保持原有资本主义制度五十年不变，具体是指哪个时间段？</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>【依据】《香港特别行政区基本法》第五条 基本法第五条明确规定，香港保持原有资本主义制度和生活方式，五十年不变，即自1997年起至2047年止。</t>
+          <t>依据：《香港特别行政区基本法》第五条。基本法第五条明确规定，香港保持原有资本主义制度和生活方式，五十年不变，即自1997年起至2047年止。</t>
         </is>
       </c>
     </row>
@@ -671,14 +671,14 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>【依据】历史记录 董建华于1997年7月1日就任香港特别行政区首任行政长官，任期至2005年。</t>
+          <t>依据：历史记录。董建华于1997年7月1日就任香港特别行政区首任行政长官，任期至2005年。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>《中英联合声明》的主要内容包括以下哪些？（多选）[多选题]</t>
+          <t>《中英联合声明》的主要内容包括以下哪些？(ABC)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>香港回归后实行"一国两制"，保持现行制度五十年不变</t>
+          <t>香港回归后实行一国两制，保持现行制度五十年不变</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -708,14 +708,14 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>【依据】《中英联合声明》（1984年） 联合声明确立了主权移交时间、"一国两制"政策及制度不变承诺。D项错误，回归后防务由中国负责，英方不保留军事基地。</t>
+          <t>依据：《中英联合声明》（1984年）。联合声明确立了主权移交时间、一国两制政策及制度不变承诺。D项错误，回归后防务由中国负责，英方不保留军事基地。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>以下关于香港特别行政区的描述，正确的是？（多选）[多选题]</t>
+          <t>以下关于香港特别行政区的描述，正确的是？(ABD)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -745,14 +745,14 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>【依据】《香港特别行政区基本法》；地理知识 香港由三大地理区域组成，位于珠江口东岸，是国际金融中心。C项错误，澳门也是特别行政区。</t>
+          <t>依据：《香港特别行政区基本法》；地理知识。香港由三大地理区域组成，位于珠江口东岸，是国际金融中心。C项错误，澳门也是特别行政区。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>根据《基本法》，以下哪些是香港特别行政区依法享有的高度自治权？（多选）[多选题]</t>
+          <t>根据《基本法》，以下哪些是香港特别行政区依法享有的高度自治权？(ABCD)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>以"中国香港"名义参与相关国际组织和活动</t>
+          <t>以中国香港名义参与相关国际组织和活动</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>【依据】《香港特别行政区基本法》第二条、第十六条、第十七条、第十九条 基本法第二条授权香港享有高度自治权，涵盖行政、立法、司法及对外事务等各方面。</t>
+          <t>依据：《香港特别行政区基本法》第二条、第十六条、第十七条、第十九条。基本法第二条授权香港享有高度自治权，涵盖行政、立法、司法及对外事务等各方面。</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>【依据】《香港特别行政区基本法》第一条 基本法第一条明确指出，香港特别行政区是中华人民共和国不可分离的部分，享有高度自治权。</t>
+          <t>依据：《香港特别行政区基本法》第一条。基本法第一条明确指出，香港特别行政区是中华人民共和国不可分离的部分，享有高度自治权。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch to latest Wenjuanxing single-cell br format for Excel import
Co-authored-by: Alanc0414 <Alanc0414@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CMport_问卷星导入_Day1.xlsx
+++ b/CMport_问卷星导入_Day1.xlsx
@@ -413,8 +413,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -422,388 +425,74 @@
           <t>题干</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>选项A</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>选项B</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>选项C</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>选项D</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>正确答案</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>解析</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>香港正式回归中国、香港特别行政区宣告成立的日期是？</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1997年6月30日</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1997年7月1日</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1999年7月1日</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1997年8月1日</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>依据：历史档案/《中英联合声明》。1997年7月1日零时，中英两国完成政权交接，中国对香港恢复行使主权，香港特别行政区正式成立。</t>
+          <t>1. 香港正式回归中国、香港特别行政区宣告成立的日期是？&lt;br/&gt;&lt;br/&gt;A. 1997年6月30日&lt;br/&gt;B. 1997年7月1日&lt;br/&gt;C. 1999年7月1日&lt;br/&gt;D. 1997年8月1日&lt;br/&gt;&lt;br/&gt;答案：B</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>中英两国政府正式签署《中英联合声明》的年份是？</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1982年</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1984年</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1986年</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1990年</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>依据：《中英联合声明》（1984年12月19日签署）。1984年12月19日，国务院总理赵紫阳与英国首相撒切尔夫人在北京签署《中英联合声明》，确定了香港回归的法律基础。</t>
+          <t>2. 中英两国政府正式签署《中英联合声明》的年份是？&lt;br/&gt;&lt;br/&gt;A. 1982年&lt;br/&gt;B. 1984年&lt;br/&gt;C. 1986年&lt;br/&gt;D. 1990年&lt;br/&gt;&lt;br/&gt;答案：B</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>一国两制伟大构想的提出者是？</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>毛泽东</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>周恩来</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>邓小平</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>江泽民</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>依据：邓小平系列讲话（1982年起）。一国两制由邓小平同志创造性提出，体现了解决历史遗留问题的政治智慧，并在香港成功实践。</t>
+          <t>3. 一国两制伟大构想的提出者是？&lt;br/&gt;&lt;br/&gt;A. 毛泽东&lt;br/&gt;B. 周恩来&lt;br/&gt;C. 邓小平&lt;br/&gt;D. 江泽民&lt;br/&gt;&lt;br/&gt;答案：C</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>香港特别行政区区旗的主体图案是什么？</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>红底白色五星</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>红底白色洋紫荆花</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>白底红色紫荆花</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>黄底红色紫荆花</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>依据：《香港特别行政区基本法》附件/区旗区徽条例。香港区旗为红底，中央绘有五星花蕊的白色洋紫荆花图案，象征香港是祖国大家庭的一员。</t>
+          <t>4. 香港特别行政区区旗的主体图案是什么？&lt;br/&gt;&lt;br/&gt;A. 红底白色五星&lt;br/&gt;B. 红底白色洋紫荆花&lt;br/&gt;C. 白底红色紫荆花&lt;br/&gt;D. 黄底红色紫荆花&lt;br/&gt;&lt;br/&gt;答案：B</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>根据《基本法》，香港保持原有资本主义制度五十年不变，具体是指哪个时间段？</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1984年至2034年</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1997年至2047年</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1990年至2040年</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>1997年至2050年</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>依据：《香港特别行政区基本法》第五条。基本法第五条明确规定，香港保持原有资本主义制度和生活方式，五十年不变，即自1997年起至2047年止。</t>
+          <t>5. 根据《基本法》，香港保持原有资本主义制度五十年不变，具体是指哪个时间段？&lt;br/&gt;&lt;br/&gt;A. 1984年至2034年&lt;br/&gt;B. 1997年至2047年&lt;br/&gt;C. 1990年至2040年&lt;br/&gt;D. 1997年至2050年&lt;br/&gt;&lt;br/&gt;答案：B</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>香港特别行政区第一任行政长官是谁？</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>曾荫权</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>梁振英</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>董建华</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>林郑月娥</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>依据：历史记录。董建华于1997年7月1日就任香港特别行政区首任行政长官，任期至2005年。</t>
+          <t>6. 香港特别行政区第一任行政长官是谁？&lt;br/&gt;&lt;br/&gt;A. 曾荫权&lt;br/&gt;B. 梁振英&lt;br/&gt;C. 董建华&lt;br/&gt;D. 林郑月娥&lt;br/&gt;&lt;br/&gt;答案：C</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>《中英联合声明》的主要内容包括以下哪些？(ABC)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>中国于1997年7月1日对香港恢复行使主权</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>英国于1997年7月1日将香港交还中国</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>香港回归后实行一国两制，保持现行制度五十年不变</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>英国可在香港保留军事基地50年</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>ABC</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>依据：《中英联合声明》（1984年）。联合声明确立了主权移交时间、一国两制政策及制度不变承诺。D项错误，回归后防务由中国负责，英方不保留军事基地。</t>
+          <t>7. 《中英联合声明》的主要内容包括以下哪些（ ）&lt;br/&gt;&lt;br/&gt;A. 中国于1997年7月1日对香港恢复行使主权&lt;br/&gt;B. 英国于1997年7月1日将香港交还中国&lt;br/&gt;C. 香港回归后实行一国两制，保持现行制度五十年不变&lt;br/&gt;D. 英国可在香港保留军事基地50年&lt;br/&gt;&lt;br/&gt;答案：ABC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>以下关于香港特别行政区的描述，正确的是？(ABD)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>香港位于中国南部，珠江口以东</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>香港由香港岛、九龙和新界三大部分组成</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>香港是中国唯一的特别行政区</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>香港是全球重要的金融、贸易及航运中心</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>ABD</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>依据：《香港特别行政区基本法》；地理知识。香港由三大地理区域组成，位于珠江口东岸，是国际金融中心。C项错误，澳门也是特别行政区。</t>
+          <t>8. 以下关于香港特别行政区的描述，正确的是（ ）&lt;br/&gt;&lt;br/&gt;A. 香港位于中国南部，珠江口以东&lt;br/&gt;B. 香港由香港岛、九龙和新界三大部分组成&lt;br/&gt;C. 香港是中国唯一的特别行政区&lt;br/&gt;D. 香港是全球重要的金融、贸易及航运中心&lt;br/&gt;&lt;br/&gt;答案：ABD</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>根据《基本法》，以下哪些是香港特别行政区依法享有的高度自治权？(ABCD)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>独立的司法权和终审权</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>行政管理权</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>立法权</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>以中国香港名义参与相关国际组织和活动</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>ABCD</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>依据：《香港特别行政区基本法》第二条、第十六条、第十七条、第十九条。基本法第二条授权香港享有高度自治权，涵盖行政、立法、司法及对外事务等各方面。</t>
+          <t>9. 根据《基本法》，以下哪些是香港特别行政区依法享有的高度自治权（ ）&lt;br/&gt;&lt;br/&gt;A. 独立的司法权和终审权&lt;br/&gt;B. 行政管理权&lt;br/&gt;C. 立法权&lt;br/&gt;D. 以中国香港名义参与相关国际组织和活动&lt;br/&gt;&lt;br/&gt;答案：ABCD</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>香港特别行政区于{1997}年{7}月{1}日正式成立，是中华人民共和国的一个享有高度自治权的{特别}行政区。</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>1997;7;1;特别</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>依据：《香港特别行政区基本法》第一条。基本法第一条明确指出，香港特别行政区是中华人民共和国不可分离的部分，享有高度自治权。</t>
+          <t>10. 香港特别行政区于____年____月____日正式成立，是中华人民共和国的一个享有高度自治权的____行政区。&lt;br/&gt;&lt;br/&gt;答案：1997；7；1；特别&lt;br/&gt;&lt;br/&gt;解析：依据：《香港特别行政区基本法》第一条。基本法第一条明确指出，香港特别行政区是中华人民共和国不可分离的部分，享有高度自治权。&lt;br/&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>